<commit_message>
📊 Actualizar VENTAS_Y_ABONOS_PF.xlsx — 14-04-2026, 2:01:47 p. m.
</commit_message>
<xml_diff>
--- a/datos/VENTAS_Y_ABONOS_PF.xlsx
+++ b/datos/VENTAS_Y_ABONOS_PF.xlsx
@@ -5,22 +5,35 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/abril/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7D9A451-D0A7-449D-ABC3-AD044F211A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB723DB7-C72C-440F-A3B2-BDE33B5254D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ParamQuery Pro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="454">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -232,6 +245,159 @@
     <t>02/05/2026</t>
   </si>
   <si>
+    <t>4246</t>
+  </si>
+  <si>
+    <t>RODRIGO IGNACIO CASTRO FIGUEROA</t>
+  </si>
+  <si>
+    <t>GARATE RIVEROS PATRICIA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>9251094-8</t>
+  </si>
+  <si>
+    <t>Los claveles, Valle de la luna, 241 - Quilicura -</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Quilicura</t>
+  </si>
+  <si>
+    <t>973063701</t>
+  </si>
+  <si>
+    <t>garateriveros2013@gmail.com</t>
+  </si>
+  <si>
+    <t>Programas de Homenajes</t>
+  </si>
+  <si>
+    <t>Raíces de Vida Libre</t>
+  </si>
+  <si>
+    <t>LIBRE</t>
+  </si>
+  <si>
+    <t>2000000</t>
+  </si>
+  <si>
+    <t>3780000</t>
+  </si>
+  <si>
+    <t>1.89</t>
+  </si>
+  <si>
+    <t>200000</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>1800000</t>
+  </si>
+  <si>
+    <t>1512605.042</t>
+  </si>
+  <si>
+    <t>-1980000</t>
+  </si>
+  <si>
+    <t>567000</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>05/05/2026</t>
+  </si>
+  <si>
+    <t>4252</t>
+  </si>
+  <si>
+    <t>ABONADO</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>WALTER FERRO</t>
+  </si>
+  <si>
+    <t>NELSON RODRIGUEZ</t>
+  </si>
+  <si>
+    <t>HUINCATRIPAI CARRASCO JUAN ALBERTO</t>
+  </si>
+  <si>
+    <t>12750788-0</t>
+  </si>
+  <si>
+    <t>José artigas, , 12432 - La Pintana -</t>
+  </si>
+  <si>
+    <t>La Pintana</t>
+  </si>
+  <si>
+    <t>934177510</t>
+  </si>
+  <si>
+    <t>ahuincatripai@gmail.com</t>
+  </si>
+  <si>
+    <t>Semillas de Legado Personal</t>
+  </si>
+  <si>
+    <t>PERSONAL</t>
+  </si>
+  <si>
+    <t>2200000</t>
+  </si>
+  <si>
+    <t>4800000</t>
+  </si>
+  <si>
+    <t>2.18</t>
+  </si>
+  <si>
+    <t>250000</t>
+  </si>
+  <si>
+    <t>11.36</t>
+  </si>
+  <si>
+    <t>1950000</t>
+  </si>
+  <si>
+    <t>-2850000</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>1166666.64</t>
+  </si>
+  <si>
+    <t>2026-04-11T00:00:00</t>
+  </si>
+  <si>
+    <t>4251</t>
+  </si>
+  <si>
+    <t>50009</t>
+  </si>
+  <si>
+    <t>CARREÑO SANTANA CAROLINA DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>11316913-3</t>
+  </si>
+  <si>
+    <t>, , 12432 - La Pintana -</t>
+  </si>
+  <si>
     <t>4174</t>
   </si>
   <si>
@@ -250,9 +416,6 @@
     <t>Augusto Villanueva , , 65 - Ñuñoa -</t>
   </si>
   <si>
-    <t>Santiago</t>
-  </si>
-  <si>
     <t>Ñuñoa</t>
   </si>
   <si>
@@ -262,9 +425,6 @@
     <t>gabrielaproteccionfamiliar@gmail.com</t>
   </si>
   <si>
-    <t>Programas de Homenajes</t>
-  </si>
-  <si>
     <t>Tesoros del Alma Siempre Juntos</t>
   </si>
   <si>
@@ -301,10 +461,79 @@
     <t>3802500</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>05/05/2026</t>
+    <t>4204</t>
+  </si>
+  <si>
+    <t>Glenda Patricia Martinez  Ortiz</t>
+  </si>
+  <si>
+    <t>TAMARA PATRICIA ARAYA MARAMBIO</t>
+  </si>
+  <si>
+    <t>JARAMILLO TAPIA PABLO</t>
+  </si>
+  <si>
+    <t>7722815-2</t>
+  </si>
+  <si>
+    <t>Santa Bárbara , , 6862 - Huechuraba -</t>
+  </si>
+  <si>
+    <t>Huechuraba</t>
+  </si>
+  <si>
+    <t>998954636</t>
+  </si>
+  <si>
+    <t>pablojaratap@gmail.com</t>
+  </si>
+  <si>
+    <t>5280000</t>
+  </si>
+  <si>
+    <t>2.4</t>
+  </si>
+  <si>
+    <t>1848739.496</t>
+  </si>
+  <si>
+    <t>-3080000</t>
+  </si>
+  <si>
+    <t>792000</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>06/05/2026</t>
+  </si>
+  <si>
+    <t>2026-04-09T00:00:00</t>
+  </si>
+  <si>
+    <t>4234</t>
+  </si>
+  <si>
+    <t>DOMINGUEZ BARRIOS MARTA ORIANA</t>
+  </si>
+  <si>
+    <t>7078549-8</t>
+  </si>
+  <si>
+    <t>Pasaje ventana , , 521 - Quilicura -</t>
+  </si>
+  <si>
+    <t>987185292</t>
+  </si>
+  <si>
+    <t>martadominguezbarrios@gmail.com</t>
+  </si>
+  <si>
+    <t>SUCURSAL</t>
+  </si>
+  <si>
+    <t>945000</t>
   </si>
   <si>
     <t>4209</t>
@@ -334,18 +563,12 @@
     <t>Tesoros del Alma Personal</t>
   </si>
   <si>
-    <t>PERSONAL</t>
-  </si>
-  <si>
     <t>3500000</t>
   </si>
   <si>
     <t>100</t>
   </si>
   <si>
-    <t>SUCURSAL</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -355,6 +578,225 @@
     <t>07/04/2026</t>
   </si>
   <si>
+    <t>4225</t>
+  </si>
+  <si>
+    <t>1059996</t>
+  </si>
+  <si>
+    <t>ROMAN DIAZ ALICIA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>5726762-3</t>
+  </si>
+  <si>
+    <t>VOLCAN TECHAU 5828, , 5828 - La Florida -</t>
+  </si>
+  <si>
+    <t>La Florida</t>
+  </si>
+  <si>
+    <t>985451468</t>
+  </si>
+  <si>
+    <t>957040801</t>
+  </si>
+  <si>
+    <t>NFMigration@funerariaim.cl</t>
+  </si>
+  <si>
+    <t>Raíces de Vida Solución Total Personal</t>
+  </si>
+  <si>
+    <t>2450000</t>
+  </si>
+  <si>
+    <t>29499900</t>
+  </si>
+  <si>
+    <t>12.04</t>
+  </si>
+  <si>
+    <t>470000</t>
+  </si>
+  <si>
+    <t>19.18</t>
+  </si>
+  <si>
+    <t>1980000</t>
+  </si>
+  <si>
+    <t>1663865.546</t>
+  </si>
+  <si>
+    <t>-27519900</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>1150003.8</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>08/04/2026</t>
+  </si>
+  <si>
+    <t>2024-12-31T00:00:00</t>
+  </si>
+  <si>
+    <t>4240</t>
+  </si>
+  <si>
+    <t>Diego Alejandro Vasquez Flores</t>
+  </si>
+  <si>
+    <t>PONCE AVENDAÑO NATALIA AMELIA</t>
+  </si>
+  <si>
+    <t>13274328-2</t>
+  </si>
+  <si>
+    <t>Pje cuarzo, , 2686 - Puente Alto -</t>
+  </si>
+  <si>
+    <t>Cordillera</t>
+  </si>
+  <si>
+    <t>Puente Alto</t>
+  </si>
+  <si>
+    <t>979961317</t>
+  </si>
+  <si>
+    <t>nataliaponce224@gmail.com</t>
+  </si>
+  <si>
+    <t>Semillas de Legado Libre</t>
+  </si>
+  <si>
+    <t>2800000</t>
+  </si>
+  <si>
+    <t>40320000</t>
+  </si>
+  <si>
+    <t>14.4</t>
+  </si>
+  <si>
+    <t>1120000</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>1680000</t>
+  </si>
+  <si>
+    <t>1411764.706</t>
+  </si>
+  <si>
+    <t>-38640000</t>
+  </si>
+  <si>
+    <t>10/05/2026</t>
+  </si>
+  <si>
+    <t>4241</t>
+  </si>
+  <si>
+    <t>4242</t>
+  </si>
+  <si>
+    <t>Daniela Andrea Rivera  Hurtado</t>
+  </si>
+  <si>
+    <t>PEREZ MONTECINOS TIHARE DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>15790568-6</t>
+  </si>
+  <si>
+    <t>Luis frez magallanes, , 926 - Puente Alto -</t>
+  </si>
+  <si>
+    <t>991401265</t>
+  </si>
+  <si>
+    <t>tihareperezm@gmail.com</t>
+  </si>
+  <si>
+    <t>2.1</t>
+  </si>
+  <si>
+    <t>400000</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>1600000</t>
+  </si>
+  <si>
+    <t>1344537.815</t>
+  </si>
+  <si>
+    <t>-2600000</t>
+  </si>
+  <si>
+    <t>490000.35</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>11/05/2026</t>
+  </si>
+  <si>
+    <t>4247</t>
+  </si>
+  <si>
+    <t>Francesca Nicole Sanchez pacheco</t>
+  </si>
+  <si>
+    <t>OJEDA HUENCHUL SANDRA YANETT</t>
+  </si>
+  <si>
+    <t>13848026-7</t>
+  </si>
+  <si>
+    <t>De lo infante , , 1987 - Maipú -</t>
+  </si>
+  <si>
+    <t>Maipú</t>
+  </si>
+  <si>
+    <t>928166556</t>
+  </si>
+  <si>
+    <t>sandraojeda2509@gmail.com</t>
+  </si>
+  <si>
+    <t>882000</t>
+  </si>
+  <si>
+    <t>0.44</t>
+  </si>
+  <si>
+    <t>1680672.269</t>
+  </si>
+  <si>
+    <t>1118000</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>874851.39</t>
+  </si>
+  <si>
     <t>4206</t>
   </si>
   <si>
@@ -370,21 +812,12 @@
     <t>, , 11180 - La Florida -</t>
   </si>
   <si>
-    <t>La Florida</t>
-  </si>
-  <si>
     <t>993332467</t>
   </si>
   <si>
     <t>hugonuñezvaldes@gmail.com</t>
   </si>
   <si>
-    <t>Raíces de Vida Solución Total Personal</t>
-  </si>
-  <si>
-    <t>2450000</t>
-  </si>
-  <si>
     <t>47775000</t>
   </si>
   <si>
@@ -424,9 +857,6 @@
     <t>Raíces de Vida Personal</t>
   </si>
   <si>
-    <t>1800000</t>
-  </si>
-  <si>
     <t>38610000</t>
   </si>
   <si>
@@ -445,6 +875,60 @@
     <t>-37440000</t>
   </si>
   <si>
+    <t>4262</t>
+  </si>
+  <si>
+    <t>80000</t>
+  </si>
+  <si>
+    <t>JORQUERA ALVAREZ MARIA FABIOLA</t>
+  </si>
+  <si>
+    <t>10323890-0</t>
+  </si>
+  <si>
+    <t>VOLCAN POMERAPE, ALT 154 - San Bernardo -</t>
+  </si>
+  <si>
+    <t>Maipo</t>
+  </si>
+  <si>
+    <t>San Bernardo</t>
+  </si>
+  <si>
+    <t>961018457</t>
+  </si>
+  <si>
+    <t>BRIDGEMATTA@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>Semillas de Legado Solución Total Libre</t>
+  </si>
+  <si>
+    <t>LIBRE SOLUCIÓN TOTAL</t>
+  </si>
+  <si>
+    <t>3450000</t>
+  </si>
+  <si>
+    <t>345000</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>3105000</t>
+  </si>
+  <si>
+    <t>1397250</t>
+  </si>
+  <si>
+    <t>15/05/2026</t>
+  </si>
+  <si>
+    <t>2026-04-14T00:00:00</t>
+  </si>
+  <si>
     <t>4176</t>
   </si>
   <si>
@@ -478,9 +962,6 @@
     <t>285000</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>2565000</t>
   </si>
   <si>
@@ -490,49 +971,82 @@
     <t>-4360500</t>
   </si>
   <si>
-    <t>36</t>
-  </si>
-  <si>
     <t>1731375</t>
   </si>
   <si>
-    <t>15/05/2026</t>
-  </si>
-  <si>
-    <t>4200</t>
-  </si>
-  <si>
-    <t>ABONADO</t>
+    <t>4250</t>
+  </si>
+  <si>
+    <t>EDIXON MANUEL BASTIDAS VASQUEZ</t>
+  </si>
+  <si>
+    <t>OYARZO LAVADO EDGARDO ANDRES</t>
+  </si>
+  <si>
+    <t>16101079-0</t>
+  </si>
+  <si>
+    <t>El belloto 10330, , 10330 - La Granja -</t>
+  </si>
+  <si>
+    <t>La Granja</t>
+  </si>
+  <si>
+    <t>977052280</t>
+  </si>
+  <si>
+    <t>edgarcrix@gmail.com</t>
+  </si>
+  <si>
+    <t>9315000</t>
+  </si>
+  <si>
+    <t>690000</t>
+  </si>
+  <si>
+    <t>2760000</t>
+  </si>
+  <si>
+    <t>2319327.731</t>
+  </si>
+  <si>
+    <t>-6555000</t>
+  </si>
+  <si>
+    <t>1811250.18</t>
+  </si>
+  <si>
+    <t>4253</t>
+  </si>
+  <si>
+    <t>PALMA CONTRERAS CARLOS JORGE</t>
+  </si>
+  <si>
+    <t>4015060-9</t>
+  </si>
+  <si>
+    <t>, , 500 - Santiago -</t>
+  </si>
+  <si>
+    <t>993001849</t>
+  </si>
+  <si>
+    <t>GFERNANDEZ@UC.CL</t>
+  </si>
+  <si>
+    <t>Semillas de Legado Solución Total Adulto Mayor</t>
+  </si>
+  <si>
+    <t>ADULTO MAYOR SOLUCIÓN TOTAL</t>
+  </si>
+  <si>
+    <t>3150000</t>
   </si>
   <si>
     <t>283500</t>
   </si>
   <si>
-    <t>PALMA CONTRERAS CARLOS JORGE</t>
-  </si>
-  <si>
-    <t>4015060-9</t>
-  </si>
-  <si>
-    <t>, , 500 - Santiago -</t>
-  </si>
-  <si>
-    <t>993001849</t>
-  </si>
-  <si>
-    <t>GFERNANDEZ@UC.CL</t>
-  </si>
-  <si>
-    <t>Semillas de Legado Solución Total Adulto Mayor</t>
-  </si>
-  <si>
-    <t>ADULTO MAYOR SOLUCIÓN TOTAL</t>
-  </si>
-  <si>
-    <t>3150000</t>
-  </si>
-  <si>
-    <t>7641000</t>
+    <t>0.09</t>
   </si>
   <si>
     <t>315000</t>
@@ -544,13 +1058,13 @@
     <t>2382352.941</t>
   </si>
   <si>
-    <t>-4806000</t>
+    <t>2551500</t>
   </si>
   <si>
     <t>12</t>
   </si>
   <si>
-    <t>5741999.82</t>
+    <t>5740875</t>
   </si>
   <si>
     <t>17</t>
@@ -559,9 +1073,6 @@
     <t>17/05/2026</t>
   </si>
   <si>
-    <t>2026-04-07T00:00:00</t>
-  </si>
-  <si>
     <t>4197</t>
   </si>
   <si>
@@ -574,9 +1085,6 @@
     <t>ALFREDO SANTANDER, , 1539 - Quilicura -</t>
   </si>
   <si>
-    <t>Quilicura</t>
-  </si>
-  <si>
     <t>988574499</t>
   </si>
   <si>
@@ -592,9 +1100,6 @@
     <t>570000</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>2280000</t>
   </si>
   <si>
@@ -631,30 +1136,18 @@
     <t>EL RELATO 2304 F 306, , 2304 - Puente Alto -</t>
   </si>
   <si>
-    <t>Cordillera</t>
-  </si>
-  <si>
-    <t>Puente Alto</t>
-  </si>
-  <si>
     <t>992589751</t>
   </si>
   <si>
     <t>934945738</t>
   </si>
   <si>
-    <t>NFMigration@funerariaim.cl</t>
-  </si>
-  <si>
     <t>27000120</t>
   </si>
   <si>
     <t>11.02</t>
   </si>
   <si>
-    <t>50000</t>
-  </si>
-  <si>
     <t>2.04</t>
   </si>
   <si>
@@ -682,9 +1175,6 @@
     <t>4214</t>
   </si>
   <si>
-    <t>WALTER FERRO</t>
-  </si>
-  <si>
     <t>MARCELO CISTERNA LEON</t>
   </si>
   <si>
@@ -697,9 +1187,6 @@
     <t>, Jardines de Rinconada, 2321 - Maipú -</t>
   </si>
   <si>
-    <t>Maipú</t>
-  </si>
-  <si>
     <t>975878952</t>
   </si>
   <si>
@@ -721,9 +1208,6 @@
     <t>11.76</t>
   </si>
   <si>
-    <t>200000</t>
-  </si>
-  <si>
     <t>5.88</t>
   </si>
   <si>
@@ -736,9 +1220,6 @@
     <t>-36800000</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>4000000</t>
   </si>
   <si>
@@ -748,6 +1229,105 @@
     <t>25/04/2026</t>
   </si>
   <si>
+    <t>4233</t>
+  </si>
+  <si>
+    <t>VILLALOBOS CONCHA ERICO RICARDO</t>
+  </si>
+  <si>
+    <t>9491090-0</t>
+  </si>
+  <si>
+    <t>Santa Elena, , 309 - Puente Alto -</t>
+  </si>
+  <si>
+    <t>999119779</t>
+  </si>
+  <si>
+    <t>ricardo.villalobos.c@gmail.com</t>
+  </si>
+  <si>
+    <t>16800000</t>
+  </si>
+  <si>
+    <t>8.4</t>
+  </si>
+  <si>
+    <t>300000</t>
+  </si>
+  <si>
+    <t>1700000</t>
+  </si>
+  <si>
+    <t>1428571.429</t>
+  </si>
+  <si>
+    <t>-15100000</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>6300000</t>
+  </si>
+  <si>
+    <t>25/05/2026</t>
+  </si>
+  <si>
+    <t>4223</t>
+  </si>
+  <si>
+    <t>SILVA VALDES LUIS FERNANDO</t>
+  </si>
+  <si>
+    <t>6675889-3</t>
+  </si>
+  <si>
+    <t>lo bascuñan 664, , 664 - Quilicura -</t>
+  </si>
+  <si>
+    <t>997224476</t>
+  </si>
+  <si>
+    <t>nfmigration@funerariaim.cl</t>
+  </si>
+  <si>
+    <t>18300000</t>
+  </si>
+  <si>
+    <t>7.47</t>
+  </si>
+  <si>
+    <t>-16320000</t>
+  </si>
+  <si>
+    <t>1522222.2</t>
+  </si>
+  <si>
+    <t>27/04/2026</t>
+  </si>
+  <si>
+    <t>4263</t>
+  </si>
+  <si>
+    <t>0.02</t>
+  </si>
+  <si>
+    <t>2899159.664</t>
+  </si>
+  <si>
+    <t>3370000</t>
+  </si>
+  <si>
+    <t>1935957.456</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>29/05/2026</t>
+  </si>
+  <si>
     <t>4195</t>
   </si>
   <si>
@@ -796,9 +1376,6 @@
     <t>4175</t>
   </si>
   <si>
-    <t>Daniela Andrea Rivera  Hurtado</t>
-  </si>
-  <si>
     <t>MARTINEZ CONTRERAS RICHARD OMAR</t>
   </si>
   <si>
@@ -812,21 +1389,6 @@
   </si>
   <si>
     <t>ecommerce.richardmartinez11@gmail.com</t>
-  </si>
-  <si>
-    <t>Raíces de Vida Libre</t>
-  </si>
-  <si>
-    <t>LIBRE</t>
-  </si>
-  <si>
-    <t>2000000</t>
-  </si>
-  <si>
-    <t>2.1</t>
-  </si>
-  <si>
-    <t>1512605.042</t>
   </si>
   <si>
     <t>-2400000</t>
@@ -1693,11 +2255,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM13"/>
+  <dimension ref="A1:AM28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="38" width="8" customWidth="1"/>
-    <col min="39" max="39" width="15" customWidth="1"/>
+    <col min="1" max="39" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" x14ac:dyDescent="0.3">
@@ -1958,91 +2519,91 @@
         <v>44</v>
       </c>
       <c r="G3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" t="s">
         <v>72</v>
       </c>
-      <c r="I3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>73</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>74</v>
-      </c>
-      <c r="L3" t="s">
-        <v>75</v>
       </c>
       <c r="M3" t="s">
         <v>51</v>
       </c>
       <c r="N3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O3" t="s">
         <v>76</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q3" t="s">
         <v>77</v>
       </c>
-      <c r="P3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>78</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>79</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>80</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>81</v>
-      </c>
-      <c r="U3" t="s">
-        <v>82</v>
       </c>
       <c r="V3" t="s">
         <v>59</v>
       </c>
       <c r="W3" t="s">
+        <v>82</v>
+      </c>
+      <c r="X3" t="s">
         <v>83</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Y3" t="s">
         <v>84</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>85</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>86</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
         <v>87</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AC3" t="s">
         <v>88</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>89</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>90</v>
       </c>
       <c r="AE3" t="s">
         <v>65</v>
       </c>
       <c r="AF3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH3" t="s">
         <v>91</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AI3" t="s">
         <v>92</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>94</v>
       </c>
       <c r="AJ3" t="s">
         <v>47</v>
@@ -2062,106 +2623,106 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" t="s">
         <v>95</v>
       </c>
-      <c r="C4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G4" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I4" t="s">
         <v>47</v>
       </c>
       <c r="J4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M4" t="s">
         <v>51</v>
       </c>
       <c r="N4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P4" t="s">
-        <v>101</v>
+        <v>47</v>
       </c>
       <c r="Q4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="V4" t="s">
         <v>59</v>
       </c>
       <c r="W4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X4" t="s">
-        <v>42</v>
+        <v>107</v>
       </c>
       <c r="Y4" t="s">
-        <v>42</v>
+        <v>108</v>
       </c>
       <c r="Z4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="AA4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="AB4" t="s">
-        <v>42</v>
+        <v>111</v>
       </c>
       <c r="AC4" t="s">
-        <v>42</v>
+        <v>111</v>
       </c>
       <c r="AD4" t="s">
-        <v>42</v>
+        <v>112</v>
       </c>
       <c r="AE4" t="s">
-        <v>107</v>
+        <v>65</v>
       </c>
       <c r="AF4" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="AG4" t="s">
-        <v>42</v>
+        <v>114</v>
       </c>
       <c r="AH4" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="AI4" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="AJ4" t="s">
         <v>47</v>
@@ -2173,7 +2734,7 @@
         <v>47</v>
       </c>
       <c r="AM4" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.3">
@@ -2181,13 +2742,13 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="E5" t="s">
         <v>43</v>
@@ -2196,91 +2757,91 @@
         <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="H5" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="I5" t="s">
         <v>47</v>
       </c>
       <c r="J5" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="K5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="L5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="M5" t="s">
         <v>51</v>
       </c>
       <c r="N5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O5" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="P5" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="Q5" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="R5" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="S5" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="T5" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="U5" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="V5" t="s">
         <v>59</v>
       </c>
       <c r="W5" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="X5" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="Y5" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="Z5" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="AA5" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="AB5" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="AC5" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="AD5" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="AE5" t="s">
         <v>65</v>
       </c>
       <c r="AF5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="AG5" t="s">
-        <v>42</v>
+        <v>114</v>
       </c>
       <c r="AH5" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="AI5" t="s">
-        <v>128</v>
+        <v>92</v>
       </c>
       <c r="AJ5" t="s">
         <v>47</v>
@@ -2292,7 +2853,7 @@
         <v>47</v>
       </c>
       <c r="AM5" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.3">
@@ -2300,7 +2861,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C6" t="s">
         <v>41</v>
@@ -2315,91 +2876,91 @@
         <v>44</v>
       </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="H6" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="I6" t="s">
         <v>47</v>
       </c>
       <c r="J6" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="K6" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="L6" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="M6" t="s">
         <v>51</v>
       </c>
       <c r="N6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O6" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="P6" t="s">
-        <v>132</v>
+        <v>47</v>
       </c>
       <c r="Q6" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="R6" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="S6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T6" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="U6" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="V6" t="s">
         <v>59</v>
       </c>
       <c r="W6" t="s">
+        <v>132</v>
+      </c>
+      <c r="X6" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y6" t="s">
         <v>134</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Z6" t="s">
         <v>135</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="AA6" t="s">
         <v>136</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AB6" t="s">
         <v>137</v>
       </c>
-      <c r="AA6" t="s">
-        <v>87</v>
-      </c>
-      <c r="AB6" t="s">
+      <c r="AC6" t="s">
         <v>138</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>139</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>140</v>
       </c>
       <c r="AE6" t="s">
         <v>65</v>
       </c>
       <c r="AF6" t="s">
-        <v>108</v>
+        <v>140</v>
       </c>
       <c r="AG6" t="s">
-        <v>42</v>
+        <v>141</v>
       </c>
       <c r="AH6" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="AI6" t="s">
-        <v>128</v>
+        <v>92</v>
       </c>
       <c r="AJ6" t="s">
         <v>47</v>
@@ -2419,13 +2980,13 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>85</v>
       </c>
       <c r="E7" t="s">
         <v>43</v>
@@ -2434,103 +2995,103 @@
         <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>143</v>
       </c>
       <c r="H7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I7" t="s">
         <v>47</v>
       </c>
       <c r="J7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="K7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="M7" t="s">
         <v>51</v>
       </c>
       <c r="N7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O7" t="s">
-        <v>76</v>
+        <v>148</v>
       </c>
       <c r="P7" t="s">
-        <v>146</v>
+        <v>47</v>
       </c>
       <c r="Q7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="R7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="S7" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="T7" t="s">
-        <v>57</v>
+        <v>104</v>
       </c>
       <c r="U7" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="V7" t="s">
         <v>59</v>
       </c>
       <c r="W7" t="s">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="X7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="Y7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="Z7" t="s">
-        <v>151</v>
+        <v>42</v>
       </c>
       <c r="AA7" t="s">
-        <v>152</v>
+        <v>42</v>
       </c>
       <c r="AB7" t="s">
+        <v>106</v>
+      </c>
+      <c r="AC7" t="s">
         <v>153</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>154</v>
-      </c>
-      <c r="AD7" t="s">
-        <v>155</v>
       </c>
       <c r="AE7" t="s">
         <v>65</v>
       </c>
       <c r="AF7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH7" t="s">
         <v>156</v>
       </c>
-      <c r="AG7" t="s">
+      <c r="AI7" t="s">
         <v>157</v>
       </c>
-      <c r="AH7" t="s">
-        <v>127</v>
-      </c>
-      <c r="AI7" t="s">
+      <c r="AJ7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM7" t="s">
         <v>158</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.3">
@@ -2541,10 +3102,10 @@
         <v>159</v>
       </c>
       <c r="C8" t="s">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>161</v>
+        <v>42</v>
       </c>
       <c r="E8" t="s">
         <v>43</v>
@@ -2556,88 +3117,88 @@
         <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="I8" t="s">
         <v>47</v>
       </c>
       <c r="J8" t="s">
+        <v>160</v>
+      </c>
+      <c r="K8" t="s">
+        <v>161</v>
+      </c>
+      <c r="L8" t="s">
         <v>162</v>
-      </c>
-      <c r="K8" t="s">
-        <v>163</v>
-      </c>
-      <c r="L8" t="s">
-        <v>164</v>
       </c>
       <c r="M8" t="s">
         <v>51</v>
       </c>
       <c r="N8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O8" t="s">
         <v>76</v>
       </c>
       <c r="P8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="Q8" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="R8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="S8" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="T8" t="s">
-        <v>167</v>
+        <v>80</v>
       </c>
       <c r="U8" t="s">
-        <v>168</v>
+        <v>81</v>
       </c>
       <c r="V8" t="s">
         <v>59</v>
       </c>
       <c r="W8" t="s">
-        <v>169</v>
+        <v>82</v>
       </c>
       <c r="X8" t="s">
-        <v>170</v>
+        <v>83</v>
       </c>
       <c r="Y8" t="s">
-        <v>150</v>
+        <v>84</v>
       </c>
       <c r="Z8" t="s">
-        <v>171</v>
+        <v>85</v>
       </c>
       <c r="AA8" t="s">
-        <v>152</v>
+        <v>86</v>
       </c>
       <c r="AB8" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="AC8" t="s">
-        <v>173</v>
+        <v>88</v>
       </c>
       <c r="AD8" t="s">
-        <v>174</v>
+        <v>89</v>
       </c>
       <c r="AE8" t="s">
-        <v>65</v>
+        <v>165</v>
       </c>
       <c r="AF8" t="s">
-        <v>175</v>
+        <v>113</v>
       </c>
       <c r="AG8" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="AH8" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="AI8" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="AJ8" t="s">
         <v>47</v>
@@ -2649,7 +3210,7 @@
         <v>47</v>
       </c>
       <c r="AM8" t="s">
-        <v>179</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.3">
@@ -2657,7 +3218,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
@@ -2666,97 +3227,97 @@
         <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H9" t="s">
-        <v>46</v>
+        <v>168</v>
       </c>
       <c r="I9" t="s">
         <v>47</v>
       </c>
       <c r="J9" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="K9" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="L9" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="M9" t="s">
         <v>51</v>
       </c>
       <c r="N9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O9" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="P9" t="s">
-        <v>47</v>
+        <v>173</v>
       </c>
       <c r="Q9" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="R9" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="S9" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="T9" t="s">
-        <v>57</v>
+        <v>175</v>
       </c>
       <c r="U9" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="V9" t="s">
         <v>59</v>
       </c>
       <c r="W9" t="s">
-        <v>60</v>
+        <v>176</v>
       </c>
       <c r="X9" t="s">
-        <v>187</v>
+        <v>42</v>
       </c>
       <c r="Y9" t="s">
-        <v>188</v>
+        <v>42</v>
       </c>
       <c r="Z9" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="AA9" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="AB9" t="s">
-        <v>191</v>
+        <v>42</v>
       </c>
       <c r="AC9" t="s">
-        <v>192</v>
+        <v>42</v>
       </c>
       <c r="AD9" t="s">
-        <v>193</v>
+        <v>42</v>
       </c>
       <c r="AE9" t="s">
-        <v>65</v>
+        <v>165</v>
       </c>
       <c r="AF9" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="AG9" t="s">
-        <v>195</v>
+        <v>42</v>
       </c>
       <c r="AH9" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="AI9" t="s">
-        <v>197</v>
+        <v>180</v>
       </c>
       <c r="AJ9" t="s">
         <v>47</v>
@@ -2776,13 +3337,13 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>198</v>
+        <v>181</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>182</v>
       </c>
       <c r="E10" t="s">
         <v>47</v>
@@ -2794,43 +3355,43 @@
         <v>47</v>
       </c>
       <c r="H10" t="s">
-        <v>199</v>
+        <v>168</v>
       </c>
       <c r="I10" t="s">
         <v>47</v>
       </c>
       <c r="J10" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="K10" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
       <c r="L10" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="M10" t="s">
         <v>51</v>
       </c>
       <c r="N10" t="s">
-        <v>203</v>
+        <v>75</v>
       </c>
       <c r="O10" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="P10" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="Q10" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="R10" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="S10" t="s">
         <v>56</v>
       </c>
       <c r="T10" t="s">
-        <v>119</v>
+        <v>190</v>
       </c>
       <c r="U10" t="s">
         <v>58</v>
@@ -2839,43 +3400,43 @@
         <v>59</v>
       </c>
       <c r="W10" t="s">
-        <v>120</v>
+        <v>191</v>
       </c>
       <c r="X10" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="Y10" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="Z10" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="AA10" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="AB10" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="AC10" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="AD10" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="AE10" t="s">
-        <v>107</v>
+        <v>165</v>
       </c>
       <c r="AF10" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="AG10" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="AH10" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="AI10" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="AJ10" t="s">
         <v>47</v>
@@ -2887,7 +3448,7 @@
         <v>47</v>
       </c>
       <c r="AM10" t="s">
-        <v>47</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.3">
@@ -2895,7 +3456,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
@@ -2910,91 +3471,91 @@
         <v>44</v>
       </c>
       <c r="G11" t="s">
-        <v>220</v>
+        <v>96</v>
       </c>
       <c r="H11" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="I11" t="s">
         <v>47</v>
       </c>
       <c r="J11" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="K11" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="L11" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="M11" t="s">
         <v>51</v>
       </c>
       <c r="N11" t="s">
-        <v>76</v>
+        <v>209</v>
       </c>
       <c r="O11" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="P11" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="Q11" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="R11" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="S11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T11" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="U11" t="s">
-        <v>229</v>
+        <v>81</v>
       </c>
       <c r="V11" t="s">
         <v>59</v>
       </c>
       <c r="W11" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="X11" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="Y11" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="Z11" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="AA11" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="AB11" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="AC11" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="AD11" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="AE11" t="s">
         <v>65</v>
       </c>
       <c r="AF11" t="s">
-        <v>238</v>
+        <v>178</v>
       </c>
       <c r="AG11" t="s">
-        <v>239</v>
+        <v>42</v>
       </c>
       <c r="AH11" t="s">
-        <v>240</v>
+        <v>86</v>
       </c>
       <c r="AI11" t="s">
-        <v>241</v>
+        <v>222</v>
       </c>
       <c r="AJ11" t="s">
         <v>47</v>
@@ -3014,7 +3575,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>242</v>
+        <v>223</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -3029,91 +3590,91 @@
         <v>44</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
       <c r="H12" t="s">
-        <v>243</v>
+        <v>205</v>
       </c>
       <c r="I12" t="s">
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="K12" t="s">
-        <v>245</v>
+        <v>207</v>
       </c>
       <c r="L12" t="s">
-        <v>246</v>
+        <v>208</v>
       </c>
       <c r="M12" t="s">
         <v>51</v>
       </c>
       <c r="N12" t="s">
-        <v>76</v>
+        <v>209</v>
       </c>
       <c r="O12" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
       <c r="P12" t="s">
-        <v>247</v>
+        <v>211</v>
       </c>
       <c r="Q12" t="s">
-        <v>247</v>
+        <v>211</v>
       </c>
       <c r="R12" t="s">
-        <v>248</v>
+        <v>212</v>
       </c>
       <c r="S12" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="T12" t="s">
-        <v>57</v>
+        <v>213</v>
       </c>
       <c r="U12" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="V12" t="s">
         <v>59</v>
       </c>
       <c r="W12" t="s">
-        <v>60</v>
+        <v>214</v>
       </c>
       <c r="X12" t="s">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="Y12" t="s">
-        <v>250</v>
+        <v>216</v>
       </c>
       <c r="Z12" t="s">
-        <v>251</v>
+        <v>217</v>
       </c>
       <c r="AA12" t="s">
-        <v>87</v>
+        <v>218</v>
       </c>
       <c r="AB12" t="s">
-        <v>252</v>
+        <v>219</v>
       </c>
       <c r="AC12" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
       <c r="AD12" t="s">
-        <v>254</v>
+        <v>221</v>
       </c>
       <c r="AE12" t="s">
         <v>65</v>
       </c>
       <c r="AF12" t="s">
-        <v>108</v>
+        <v>178</v>
       </c>
       <c r="AG12" t="s">
         <v>42</v>
       </c>
       <c r="AH12" t="s">
-        <v>255</v>
+        <v>86</v>
       </c>
       <c r="AI12" t="s">
-        <v>256</v>
+        <v>222</v>
       </c>
       <c r="AJ12" t="s">
         <v>47</v>
@@ -3133,7 +3694,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>257</v>
+        <v>224</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -3148,76 +3709,76 @@
         <v>44</v>
       </c>
       <c r="G13" t="s">
-        <v>220</v>
+        <v>96</v>
       </c>
       <c r="H13" t="s">
-        <v>258</v>
+        <v>225</v>
       </c>
       <c r="I13" t="s">
         <v>47</v>
       </c>
       <c r="J13" t="s">
-        <v>259</v>
+        <v>226</v>
       </c>
       <c r="K13" t="s">
-        <v>260</v>
+        <v>227</v>
       </c>
       <c r="L13" t="s">
-        <v>261</v>
+        <v>228</v>
       </c>
       <c r="M13" t="s">
         <v>51</v>
       </c>
       <c r="N13" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="O13" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="P13" t="s">
-        <v>262</v>
+        <v>229</v>
       </c>
       <c r="Q13" t="s">
-        <v>262</v>
+        <v>229</v>
       </c>
       <c r="R13" t="s">
-        <v>263</v>
+        <v>230</v>
       </c>
       <c r="S13" t="s">
+        <v>79</v>
+      </c>
+      <c r="T13" t="s">
         <v>80</v>
       </c>
-      <c r="T13" t="s">
-        <v>264</v>
-      </c>
       <c r="U13" t="s">
-        <v>265</v>
+        <v>81</v>
       </c>
       <c r="V13" t="s">
         <v>59</v>
       </c>
       <c r="W13" t="s">
-        <v>266</v>
+        <v>82</v>
       </c>
       <c r="X13" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="Y13" t="s">
-        <v>267</v>
+        <v>231</v>
       </c>
       <c r="Z13" t="s">
+        <v>232</v>
+      </c>
+      <c r="AA13" t="s">
         <v>233</v>
       </c>
-      <c r="AA13" t="s">
-        <v>152</v>
-      </c>
       <c r="AB13" t="s">
-        <v>134</v>
+        <v>234</v>
       </c>
       <c r="AC13" t="s">
-        <v>268</v>
+        <v>235</v>
       </c>
       <c r="AD13" t="s">
-        <v>269</v>
+        <v>236</v>
       </c>
       <c r="AE13" t="s">
         <v>65</v>
@@ -3226,24 +3787,1809 @@
         <v>66</v>
       </c>
       <c r="AG13" t="s">
+        <v>237</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>238</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>239</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>240</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" t="s">
+        <v>96</v>
+      </c>
+      <c r="H14" t="s">
+        <v>241</v>
+      </c>
+      <c r="I14" t="s">
+        <v>47</v>
+      </c>
+      <c r="J14" t="s">
+        <v>242</v>
+      </c>
+      <c r="K14" t="s">
+        <v>243</v>
+      </c>
+      <c r="L14" t="s">
+        <v>244</v>
+      </c>
+      <c r="M14" t="s">
+        <v>51</v>
+      </c>
+      <c r="N14" t="s">
+        <v>75</v>
+      </c>
+      <c r="O14" t="s">
+        <v>245</v>
+      </c>
+      <c r="P14" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>246</v>
+      </c>
+      <c r="R14" t="s">
+        <v>247</v>
+      </c>
+      <c r="S14" t="s">
+        <v>79</v>
+      </c>
+      <c r="T14" t="s">
+        <v>80</v>
+      </c>
+      <c r="U14" t="s">
+        <v>81</v>
+      </c>
+      <c r="V14" t="s">
+        <v>59</v>
+      </c>
+      <c r="W14" t="s">
+        <v>82</v>
+      </c>
+      <c r="X14" t="s">
+        <v>248</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>249</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>250</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>251</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>252</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>238</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>239</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>254</v>
+      </c>
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" t="s">
+        <v>122</v>
+      </c>
+      <c r="H15" t="s">
+        <v>255</v>
+      </c>
+      <c r="I15" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" t="s">
+        <v>256</v>
+      </c>
+      <c r="K15" t="s">
+        <v>257</v>
+      </c>
+      <c r="L15" t="s">
+        <v>258</v>
+      </c>
+      <c r="M15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N15" t="s">
+        <v>75</v>
+      </c>
+      <c r="O15" t="s">
+        <v>186</v>
+      </c>
+      <c r="P15" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>259</v>
+      </c>
+      <c r="R15" t="s">
+        <v>260</v>
+      </c>
+      <c r="S15" t="s">
+        <v>56</v>
+      </c>
+      <c r="T15" t="s">
+        <v>190</v>
+      </c>
+      <c r="U15" t="s">
+        <v>58</v>
+      </c>
+      <c r="V15" t="s">
+        <v>59</v>
+      </c>
+      <c r="W15" t="s">
+        <v>191</v>
+      </c>
+      <c r="X15" t="s">
+        <v>261</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>262</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>263</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>265</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>266</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>178</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>268</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>269</v>
+      </c>
+      <c r="C16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" t="s">
+        <v>255</v>
+      </c>
+      <c r="I16" t="s">
+        <v>47</v>
+      </c>
+      <c r="J16" t="s">
         <v>270</v>
       </c>
-      <c r="AH13" t="s">
-        <v>255</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>256</v>
-      </c>
-      <c r="AJ13" t="s">
-        <v>47</v>
-      </c>
-      <c r="AK13" t="s">
-        <v>47</v>
-      </c>
-      <c r="AL13" t="s">
-        <v>47</v>
-      </c>
-      <c r="AM13" t="s">
+      <c r="K16" t="s">
+        <v>271</v>
+      </c>
+      <c r="L16" t="s">
+        <v>258</v>
+      </c>
+      <c r="M16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N16" t="s">
+        <v>75</v>
+      </c>
+      <c r="O16" t="s">
+        <v>186</v>
+      </c>
+      <c r="P16" t="s">
+        <v>272</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>259</v>
+      </c>
+      <c r="R16" t="s">
+        <v>260</v>
+      </c>
+      <c r="S16" t="s">
+        <v>79</v>
+      </c>
+      <c r="T16" t="s">
+        <v>273</v>
+      </c>
+      <c r="U16" t="s">
+        <v>105</v>
+      </c>
+      <c r="V16" t="s">
+        <v>59</v>
+      </c>
+      <c r="W16" t="s">
+        <v>87</v>
+      </c>
+      <c r="X16" t="s">
+        <v>274</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>275</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>276</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>277</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>278</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>279</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>178</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>268</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>280</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" t="s">
+        <v>281</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" t="s">
+        <v>97</v>
+      </c>
+      <c r="I17" t="s">
+        <v>47</v>
+      </c>
+      <c r="J17" t="s">
+        <v>282</v>
+      </c>
+      <c r="K17" t="s">
+        <v>283</v>
+      </c>
+      <c r="L17" t="s">
+        <v>284</v>
+      </c>
+      <c r="M17" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" t="s">
+        <v>285</v>
+      </c>
+      <c r="O17" t="s">
+        <v>286</v>
+      </c>
+      <c r="P17" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>287</v>
+      </c>
+      <c r="R17" t="s">
+        <v>288</v>
+      </c>
+      <c r="S17" t="s">
+        <v>56</v>
+      </c>
+      <c r="T17" t="s">
+        <v>289</v>
+      </c>
+      <c r="U17" t="s">
+        <v>290</v>
+      </c>
+      <c r="V17" t="s">
+        <v>59</v>
+      </c>
+      <c r="W17" t="s">
+        <v>291</v>
+      </c>
+      <c r="X17" t="s">
+        <v>292</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>293</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>291</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>291</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>294</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>295</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>296</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="18" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>298</v>
+      </c>
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" t="s">
+        <v>299</v>
+      </c>
+      <c r="I18" t="s">
+        <v>47</v>
+      </c>
+      <c r="J18" t="s">
+        <v>300</v>
+      </c>
+      <c r="K18" t="s">
+        <v>301</v>
+      </c>
+      <c r="L18" t="s">
+        <v>302</v>
+      </c>
+      <c r="M18" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" t="s">
+        <v>75</v>
+      </c>
+      <c r="O18" t="s">
+        <v>75</v>
+      </c>
+      <c r="P18" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>304</v>
+      </c>
+      <c r="R18" t="s">
+        <v>305</v>
+      </c>
+      <c r="S18" t="s">
+        <v>56</v>
+      </c>
+      <c r="T18" t="s">
+        <v>57</v>
+      </c>
+      <c r="U18" t="s">
+        <v>58</v>
+      </c>
+      <c r="V18" t="s">
+        <v>59</v>
+      </c>
+      <c r="W18" t="s">
+        <v>60</v>
+      </c>
+      <c r="X18" t="s">
+        <v>306</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>307</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>308</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>309</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>310</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>311</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>312</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>296</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
+        <v>313</v>
+      </c>
+      <c r="C19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" t="s">
+        <v>314</v>
+      </c>
+      <c r="I19" t="s">
+        <v>47</v>
+      </c>
+      <c r="J19" t="s">
+        <v>315</v>
+      </c>
+      <c r="K19" t="s">
+        <v>316</v>
+      </c>
+      <c r="L19" t="s">
+        <v>317</v>
+      </c>
+      <c r="M19" t="s">
+        <v>51</v>
+      </c>
+      <c r="N19" t="s">
+        <v>75</v>
+      </c>
+      <c r="O19" t="s">
+        <v>318</v>
+      </c>
+      <c r="P19" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>319</v>
+      </c>
+      <c r="R19" t="s">
+        <v>320</v>
+      </c>
+      <c r="S19" t="s">
+        <v>56</v>
+      </c>
+      <c r="T19" t="s">
+        <v>289</v>
+      </c>
+      <c r="U19" t="s">
+        <v>290</v>
+      </c>
+      <c r="V19" t="s">
+        <v>59</v>
+      </c>
+      <c r="W19" t="s">
+        <v>291</v>
+      </c>
+      <c r="X19" t="s">
+        <v>321</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>322</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>323</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>324</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>325</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>326</v>
+      </c>
+      <c r="AH19" t="s">
+        <v>267</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>296</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" t="s">
+        <v>327</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" t="s">
+        <v>43</v>
+      </c>
+      <c r="F20" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" t="s">
+        <v>299</v>
+      </c>
+      <c r="I20" t="s">
+        <v>47</v>
+      </c>
+      <c r="J20" t="s">
+        <v>328</v>
+      </c>
+      <c r="K20" t="s">
+        <v>329</v>
+      </c>
+      <c r="L20" t="s">
+        <v>330</v>
+      </c>
+      <c r="M20" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" t="s">
+        <v>75</v>
+      </c>
+      <c r="O20" t="s">
+        <v>75</v>
+      </c>
+      <c r="P20" t="s">
+        <v>331</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>304</v>
+      </c>
+      <c r="R20" t="s">
+        <v>332</v>
+      </c>
+      <c r="S20" t="s">
+        <v>56</v>
+      </c>
+      <c r="T20" t="s">
+        <v>333</v>
+      </c>
+      <c r="U20" t="s">
+        <v>334</v>
+      </c>
+      <c r="V20" t="s">
+        <v>59</v>
+      </c>
+      <c r="W20" t="s">
+        <v>335</v>
+      </c>
+      <c r="X20" t="s">
+        <v>336</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>338</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>339</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>340</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>341</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>342</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>343</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>344</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>345</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s">
+        <v>346</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" t="s">
+        <v>43</v>
+      </c>
+      <c r="F21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H21" t="s">
+        <v>46</v>
+      </c>
+      <c r="I21" t="s">
+        <v>47</v>
+      </c>
+      <c r="J21" t="s">
+        <v>347</v>
+      </c>
+      <c r="K21" t="s">
+        <v>348</v>
+      </c>
+      <c r="L21" t="s">
+        <v>349</v>
+      </c>
+      <c r="M21" t="s">
+        <v>51</v>
+      </c>
+      <c r="N21" t="s">
+        <v>75</v>
+      </c>
+      <c r="O21" t="s">
+        <v>76</v>
+      </c>
+      <c r="P21" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>350</v>
+      </c>
+      <c r="R21" t="s">
+        <v>351</v>
+      </c>
+      <c r="S21" t="s">
+        <v>56</v>
+      </c>
+      <c r="T21" t="s">
+        <v>57</v>
+      </c>
+      <c r="U21" t="s">
+        <v>58</v>
+      </c>
+      <c r="V21" t="s">
+        <v>59</v>
+      </c>
+      <c r="W21" t="s">
+        <v>60</v>
+      </c>
+      <c r="X21" t="s">
+        <v>352</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>353</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>354</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>355</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>356</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>357</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>358</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>359</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>360</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>361</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
+        <v>362</v>
+      </c>
+      <c r="C22" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" t="s">
+        <v>47</v>
+      </c>
+      <c r="H22" t="s">
+        <v>363</v>
+      </c>
+      <c r="I22" t="s">
+        <v>47</v>
+      </c>
+      <c r="J22" t="s">
+        <v>364</v>
+      </c>
+      <c r="K22" t="s">
+        <v>365</v>
+      </c>
+      <c r="L22" t="s">
+        <v>366</v>
+      </c>
+      <c r="M22" t="s">
+        <v>51</v>
+      </c>
+      <c r="N22" t="s">
+        <v>209</v>
+      </c>
+      <c r="O22" t="s">
+        <v>210</v>
+      </c>
+      <c r="P22" t="s">
+        <v>367</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>368</v>
+      </c>
+      <c r="R22" t="s">
+        <v>189</v>
+      </c>
+      <c r="S22" t="s">
+        <v>56</v>
+      </c>
+      <c r="T22" t="s">
+        <v>190</v>
+      </c>
+      <c r="U22" t="s">
+        <v>58</v>
+      </c>
+      <c r="V22" t="s">
+        <v>59</v>
+      </c>
+      <c r="W22" t="s">
+        <v>191</v>
+      </c>
+      <c r="X22" t="s">
+        <v>369</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>370</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>371</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>372</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>373</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>374</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>375</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>376</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>377</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>378</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" t="s">
+        <v>379</v>
+      </c>
+      <c r="C23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" t="s">
+        <v>42</v>
+      </c>
+      <c r="E23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F23" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" t="s">
+        <v>380</v>
+      </c>
+      <c r="I23" t="s">
+        <v>47</v>
+      </c>
+      <c r="J23" t="s">
+        <v>381</v>
+      </c>
+      <c r="K23" t="s">
+        <v>382</v>
+      </c>
+      <c r="L23" t="s">
+        <v>383</v>
+      </c>
+      <c r="M23" t="s">
+        <v>51</v>
+      </c>
+      <c r="N23" t="s">
+        <v>75</v>
+      </c>
+      <c r="O23" t="s">
+        <v>245</v>
+      </c>
+      <c r="P23" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>384</v>
+      </c>
+      <c r="R23" t="s">
+        <v>385</v>
+      </c>
+      <c r="S23" t="s">
+        <v>79</v>
+      </c>
+      <c r="T23" t="s">
+        <v>386</v>
+      </c>
+      <c r="U23" t="s">
+        <v>387</v>
+      </c>
+      <c r="V23" t="s">
+        <v>59</v>
+      </c>
+      <c r="W23" t="s">
+        <v>388</v>
+      </c>
+      <c r="X23" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>390</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>392</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>394</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>156</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>395</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>396</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" t="s">
+        <v>398</v>
+      </c>
+      <c r="C24" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24" t="s">
+        <v>44</v>
+      </c>
+      <c r="G24" t="s">
+        <v>96</v>
+      </c>
+      <c r="H24" t="s">
+        <v>205</v>
+      </c>
+      <c r="I24" t="s">
+        <v>47</v>
+      </c>
+      <c r="J24" t="s">
+        <v>399</v>
+      </c>
+      <c r="K24" t="s">
+        <v>400</v>
+      </c>
+      <c r="L24" t="s">
+        <v>401</v>
+      </c>
+      <c r="M24" t="s">
+        <v>51</v>
+      </c>
+      <c r="N24" t="s">
+        <v>209</v>
+      </c>
+      <c r="O24" t="s">
+        <v>210</v>
+      </c>
+      <c r="P24" t="s">
+        <v>402</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>402</v>
+      </c>
+      <c r="R24" t="s">
+        <v>403</v>
+      </c>
+      <c r="S24" t="s">
+        <v>79</v>
+      </c>
+      <c r="T24" t="s">
+        <v>80</v>
+      </c>
+      <c r="U24" t="s">
+        <v>81</v>
+      </c>
+      <c r="V24" t="s">
+        <v>59</v>
+      </c>
+      <c r="W24" t="s">
+        <v>82</v>
+      </c>
+      <c r="X24" t="s">
+        <v>404</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>405</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>406</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>267</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>407</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>409</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>410</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>411</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>396</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>412</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" t="s">
+        <v>413</v>
+      </c>
+      <c r="C25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G25" t="s">
+        <v>47</v>
+      </c>
+      <c r="H25" t="s">
+        <v>168</v>
+      </c>
+      <c r="I25" t="s">
+        <v>47</v>
+      </c>
+      <c r="J25" t="s">
+        <v>414</v>
+      </c>
+      <c r="K25" t="s">
+        <v>415</v>
+      </c>
+      <c r="L25" t="s">
+        <v>416</v>
+      </c>
+      <c r="M25" t="s">
+        <v>51</v>
+      </c>
+      <c r="N25" t="s">
+        <v>75</v>
+      </c>
+      <c r="O25" t="s">
+        <v>76</v>
+      </c>
+      <c r="P25" t="s">
+        <v>417</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>417</v>
+      </c>
+      <c r="R25" t="s">
+        <v>418</v>
+      </c>
+      <c r="S25" t="s">
+        <v>56</v>
+      </c>
+      <c r="T25" t="s">
+        <v>190</v>
+      </c>
+      <c r="U25" t="s">
+        <v>58</v>
+      </c>
+      <c r="V25" t="s">
+        <v>59</v>
+      </c>
+      <c r="W25" t="s">
+        <v>191</v>
+      </c>
+      <c r="X25" t="s">
+        <v>419</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>420</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>194</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>195</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>196</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>197</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>375</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>422</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>375</v>
+      </c>
+      <c r="AI25" t="s">
+        <v>423</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK25" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL25" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" t="s">
+        <v>424</v>
+      </c>
+      <c r="C26" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" t="s">
+        <v>281</v>
+      </c>
+      <c r="E26" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" t="s">
+        <v>44</v>
+      </c>
+      <c r="G26" t="s">
+        <v>96</v>
+      </c>
+      <c r="H26" t="s">
+        <v>97</v>
+      </c>
+      <c r="I26" t="s">
+        <v>47</v>
+      </c>
+      <c r="J26" t="s">
+        <v>282</v>
+      </c>
+      <c r="K26" t="s">
+        <v>283</v>
+      </c>
+      <c r="L26" t="s">
+        <v>284</v>
+      </c>
+      <c r="M26" t="s">
+        <v>51</v>
+      </c>
+      <c r="N26" t="s">
+        <v>285</v>
+      </c>
+      <c r="O26" t="s">
+        <v>286</v>
+      </c>
+      <c r="P26" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>287</v>
+      </c>
+      <c r="R26" t="s">
+        <v>288</v>
+      </c>
+      <c r="S26" t="s">
+        <v>56</v>
+      </c>
+      <c r="T26" t="s">
+        <v>289</v>
+      </c>
+      <c r="U26" t="s">
+        <v>290</v>
+      </c>
+      <c r="V26" t="s">
+        <v>59</v>
+      </c>
+      <c r="W26" t="s">
+        <v>291</v>
+      </c>
+      <c r="X26" t="s">
+        <v>281</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>425</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>291</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>426</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>427</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>252</v>
+      </c>
+      <c r="AG26" t="s">
+        <v>428</v>
+      </c>
+      <c r="AH26" t="s">
+        <v>429</v>
+      </c>
+      <c r="AI26" t="s">
+        <v>430</v>
+      </c>
+      <c r="AJ26" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK26" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL26" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM26" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="27" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27" t="s">
+        <v>431</v>
+      </c>
+      <c r="C27" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" t="s">
+        <v>43</v>
+      </c>
+      <c r="F27" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" t="s">
+        <v>45</v>
+      </c>
+      <c r="H27" t="s">
+        <v>432</v>
+      </c>
+      <c r="I27" t="s">
+        <v>47</v>
+      </c>
+      <c r="J27" t="s">
+        <v>433</v>
+      </c>
+      <c r="K27" t="s">
+        <v>434</v>
+      </c>
+      <c r="L27" t="s">
+        <v>435</v>
+      </c>
+      <c r="M27" t="s">
+        <v>51</v>
+      </c>
+      <c r="N27" t="s">
+        <v>75</v>
+      </c>
+      <c r="O27" t="s">
+        <v>76</v>
+      </c>
+      <c r="P27" t="s">
+        <v>436</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>436</v>
+      </c>
+      <c r="R27" t="s">
+        <v>437</v>
+      </c>
+      <c r="S27" t="s">
+        <v>56</v>
+      </c>
+      <c r="T27" t="s">
+        <v>57</v>
+      </c>
+      <c r="U27" t="s">
+        <v>58</v>
+      </c>
+      <c r="V27" t="s">
+        <v>59</v>
+      </c>
+      <c r="W27" t="s">
+        <v>60</v>
+      </c>
+      <c r="X27" t="s">
+        <v>438</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>440</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>441</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>442</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>443</v>
+      </c>
+      <c r="AE27" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF27" t="s">
+        <v>178</v>
+      </c>
+      <c r="AG27" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH27" t="s">
+        <v>444</v>
+      </c>
+      <c r="AI27" t="s">
+        <v>445</v>
+      </c>
+      <c r="AJ27" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK27" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL27" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM27" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" t="s">
+        <v>446</v>
+      </c>
+      <c r="C28" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" t="s">
+        <v>44</v>
+      </c>
+      <c r="G28" t="s">
+        <v>96</v>
+      </c>
+      <c r="H28" t="s">
+        <v>225</v>
+      </c>
+      <c r="I28" t="s">
+        <v>47</v>
+      </c>
+      <c r="J28" t="s">
+        <v>447</v>
+      </c>
+      <c r="K28" t="s">
+        <v>448</v>
+      </c>
+      <c r="L28" t="s">
+        <v>449</v>
+      </c>
+      <c r="M28" t="s">
+        <v>51</v>
+      </c>
+      <c r="N28" t="s">
+        <v>209</v>
+      </c>
+      <c r="O28" t="s">
+        <v>210</v>
+      </c>
+      <c r="P28" t="s">
+        <v>450</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>450</v>
+      </c>
+      <c r="R28" t="s">
+        <v>451</v>
+      </c>
+      <c r="S28" t="s">
+        <v>79</v>
+      </c>
+      <c r="T28" t="s">
+        <v>80</v>
+      </c>
+      <c r="U28" t="s">
+        <v>81</v>
+      </c>
+      <c r="V28" t="s">
+        <v>59</v>
+      </c>
+      <c r="W28" t="s">
+        <v>82</v>
+      </c>
+      <c r="X28" t="s">
+        <v>135</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>231</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC28" t="s">
+        <v>88</v>
+      </c>
+      <c r="AD28" t="s">
+        <v>452</v>
+      </c>
+      <c r="AE28" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF28" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG28" t="s">
+        <v>453</v>
+      </c>
+      <c r="AH28" t="s">
+        <v>444</v>
+      </c>
+      <c r="AI28" t="s">
+        <v>445</v>
+      </c>
+      <c r="AJ28" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK28" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL28" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM28" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>